<commit_message>
Separate corpus description from results in the validation table
Removes the Verdict column from the README table and the manifest. The table
describes the corpus — what was selected and why each study is in it — and
results across the ten belong in a single results table with the statistics
and plots, not scattered through a selection listing.

The freed column now carries "Role in the matrix", which is the question the
table should answer: why is this study here and what does it test that the
others do not.

Also normalises repository names in the manifest so it matches the README:
"other" -> UCSF Dash, "curatedMetagenomicData (Bioconductor)" ->
curatedMetagenomicData, "NCBI SRA (raw reads)" -> NCBI SRA. Sorting or
filtering the spreadsheet on a value of "other" was unhelpful.

Per-study verdicts remain in each report under validation/.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QGu9FEfMNKg2pfoiEuhDfW
</commit_message>
<xml_diff>
--- a/validation/validation-set-manifest.xlsx
+++ b/validation/validation-set-manifest.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="118">
   <si>
     <t>Run order</t>
   </si>
@@ -31,9 +31,6 @@
     <t>Status</t>
   </si>
   <si>
-    <t>Verdict</t>
-  </si>
-  <si>
     <t>Paper title</t>
   </si>
   <si>
@@ -88,9 +85,6 @@
     <t>complete</t>
   </si>
   <si>
-    <t>Partially reproduced</t>
-  </si>
-  <si>
     <t>Testing the "Grandma Hypothesis": Characterizing Skin Microbiome Diversity as a Project-Based Learning Approach to Genomics</t>
   </si>
   <si>
@@ -103,7 +97,7 @@
     <t>phyloseq .RDS (course-processed)</t>
   </si>
   <si>
-    <t>NCBI SRA (raw reads)</t>
+    <t>NCBI SRA</t>
   </si>
   <si>
     <t>PRJNA553551</t>
@@ -130,9 +124,6 @@
     <t>Basic MetaPhlAn path, end to end</t>
   </si>
   <si>
-    <t>Reproduced</t>
-  </si>
-  <si>
     <t>Colorectal Cancer and the Human Gut Microbiome: Reproducibility with Whole-Genome Shotgun Sequencing</t>
   </si>
   <si>
@@ -145,7 +136,7 @@
     <t>MetaPhlAn taxonomic profile + HUMAnN functional profile</t>
   </si>
   <si>
-    <t>curatedMetagenomicData (Bioconductor)</t>
+    <t>curatedMetagenomicData</t>
   </si>
   <si>
     <t>study_name=VogtmannE_2016; PMID=27171425</t>
@@ -367,7 +358,7 @@
     <t>OTU/ASV table (CSV/TSV/XLS)</t>
   </si>
   <si>
-    <t>other</t>
+    <t>UCSF Dash</t>
   </si>
   <si>
     <t>10.7272/Q6RX997G</t>
@@ -719,10 +710,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T11"/>
+  <dimension ref="A1:S11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:20" s="1" customFormat="1">
+    <row r="1" spans="1:19" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -780,514 +771,505 @@
       <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
-        <v>19</v>
-      </c>
     </row>
-    <row r="2" spans="1:20">
+    <row r="2" spans="1:19">
       <c r="A2">
         <v>0</v>
       </c>
       <c r="B2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" t="s">
         <v>20</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>21</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>22</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>23</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>24</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2">
+        <v>2020</v>
+      </c>
+      <c r="I2" t="s">
         <v>25</v>
       </c>
-      <c r="H2" t="s">
+      <c r="J2" t="s">
         <v>26</v>
       </c>
-      <c r="I2">
-        <v>2020</v>
-      </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>27</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>28</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>29</v>
       </c>
-      <c r="M2" t="s">
+      <c r="N2" t="s">
         <v>30</v>
       </c>
-      <c r="N2" t="s">
+      <c r="O2">
+        <v>344</v>
+      </c>
+      <c r="P2">
+        <v>128</v>
+      </c>
+      <c r="Q2">
+        <v>5</v>
+      </c>
+      <c r="R2" t="s">
         <v>31</v>
       </c>
-      <c r="O2" t="s">
+      <c r="S2" t="s">
         <v>32</v>
       </c>
-      <c r="P2">
-        <v>344</v>
-      </c>
-      <c r="Q2">
-        <v>128</v>
-      </c>
-      <c r="R2">
-        <v>5</v>
-      </c>
-      <c r="S2" t="s">
-        <v>33</v>
-      </c>
-      <c r="T2" t="s">
-        <v>34</v>
-      </c>
     </row>
-    <row r="3" spans="1:20">
+    <row r="3" spans="1:19">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" t="s">
+        <v>34</v>
+      </c>
+      <c r="D3" t="s">
         <v>35</v>
       </c>
-      <c r="C3" t="s">
+      <c r="E3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" t="s">
         <v>36</v>
       </c>
-      <c r="D3" t="s">
+      <c r="G3" t="s">
         <v>37</v>
       </c>
-      <c r="E3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F3" t="s">
+      <c r="H3">
+        <v>2016</v>
+      </c>
+      <c r="I3" t="s">
         <v>38</v>
       </c>
-      <c r="G3" t="s">
+      <c r="J3" t="s">
         <v>39</v>
       </c>
-      <c r="H3" t="s">
+      <c r="K3" t="s">
         <v>40</v>
       </c>
-      <c r="I3">
-        <v>2016</v>
-      </c>
-      <c r="J3" t="s">
+      <c r="L3" t="s">
         <v>41</v>
       </c>
-      <c r="K3" t="s">
+      <c r="M3" t="s">
         <v>42</v>
       </c>
-      <c r="L3" t="s">
+      <c r="N3" t="s">
         <v>43</v>
       </c>
-      <c r="M3" t="s">
-        <v>44</v>
-      </c>
-      <c r="N3" t="s">
-        <v>45</v>
-      </c>
-      <c r="O3" t="s">
-        <v>46</v>
+      <c r="O3">
+        <v>110</v>
       </c>
       <c r="P3">
         <v>110</v>
       </c>
       <c r="Q3">
-        <v>110</v>
-      </c>
-      <c r="R3">
         <v>1</v>
       </c>
+      <c r="R3" t="s">
+        <v>44</v>
+      </c>
       <c r="S3" t="s">
-        <v>47</v>
-      </c>
-      <c r="T3" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
-    <row r="4" spans="1:20">
+    <row r="4" spans="1:19">
       <c r="A4">
         <v>2</v>
       </c>
       <c r="B4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D4" t="s">
+        <v>47</v>
+      </c>
+      <c r="E4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F4" t="s">
         <v>49</v>
       </c>
-      <c r="C4" t="s">
-        <v>36</v>
-      </c>
-      <c r="D4" t="s">
+      <c r="G4" t="s">
         <v>50</v>
       </c>
-      <c r="E4" t="s">
+      <c r="H4">
+        <v>2020</v>
+      </c>
+      <c r="I4" t="s">
         <v>51</v>
       </c>
-      <c r="G4" t="s">
+      <c r="J4" t="s">
         <v>52</v>
       </c>
-      <c r="H4" t="s">
+      <c r="K4" t="s">
         <v>53</v>
       </c>
-      <c r="I4">
-        <v>2020</v>
-      </c>
-      <c r="J4" t="s">
+      <c r="L4" t="s">
         <v>54</v>
       </c>
-      <c r="K4" t="s">
+      <c r="M4" t="s">
         <v>55</v>
       </c>
-      <c r="L4" t="s">
+      <c r="N4" t="s">
         <v>56</v>
       </c>
-      <c r="M4" t="s">
-        <v>57</v>
-      </c>
-      <c r="N4" t="s">
-        <v>58</v>
-      </c>
-      <c r="O4" t="s">
-        <v>59</v>
-      </c>
     </row>
-    <row r="5" spans="1:20">
+    <row r="5" spans="1:19">
       <c r="A5">
         <v>3</v>
       </c>
       <c r="B5" t="s">
+        <v>57</v>
+      </c>
+      <c r="C5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" t="s">
+        <v>58</v>
+      </c>
+      <c r="E5" t="s">
+        <v>48</v>
+      </c>
+      <c r="F5" t="s">
+        <v>59</v>
+      </c>
+      <c r="G5" t="s">
         <v>60</v>
       </c>
-      <c r="C5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D5" t="s">
+      <c r="H5">
+        <v>2017</v>
+      </c>
+      <c r="I5" t="s">
         <v>61</v>
       </c>
-      <c r="E5" t="s">
-        <v>51</v>
-      </c>
-      <c r="G5" t="s">
+      <c r="J5" t="s">
+        <v>52</v>
+      </c>
+      <c r="K5" t="s">
+        <v>53</v>
+      </c>
+      <c r="L5" t="s">
         <v>62</v>
       </c>
-      <c r="H5" t="s">
+      <c r="M5" t="s">
         <v>63</v>
       </c>
-      <c r="I5">
-        <v>2017</v>
-      </c>
-      <c r="J5" t="s">
+      <c r="N5" t="s">
         <v>64</v>
       </c>
-      <c r="K5" t="s">
-        <v>55</v>
-      </c>
-      <c r="L5" t="s">
-        <v>56</v>
-      </c>
-      <c r="M5" t="s">
-        <v>65</v>
-      </c>
-      <c r="N5" t="s">
-        <v>66</v>
-      </c>
-      <c r="O5" t="s">
-        <v>67</v>
-      </c>
     </row>
-    <row r="6" spans="1:20">
+    <row r="6" spans="1:19">
       <c r="A6">
         <v>4</v>
       </c>
       <c r="B6" t="s">
+        <v>65</v>
+      </c>
+      <c r="C6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" t="s">
+        <v>66</v>
+      </c>
+      <c r="E6" t="s">
+        <v>48</v>
+      </c>
+      <c r="F6" t="s">
+        <v>67</v>
+      </c>
+      <c r="G6" t="s">
         <v>68</v>
       </c>
-      <c r="C6" t="s">
-        <v>21</v>
-      </c>
-      <c r="D6" t="s">
+      <c r="H6">
+        <v>2020</v>
+      </c>
+      <c r="I6" t="s">
         <v>69</v>
       </c>
-      <c r="E6" t="s">
-        <v>51</v>
-      </c>
-      <c r="G6" t="s">
+      <c r="J6" t="s">
         <v>70</v>
       </c>
-      <c r="H6" t="s">
+      <c r="K6" t="s">
+        <v>53</v>
+      </c>
+      <c r="L6" t="s">
         <v>71</v>
       </c>
-      <c r="I6">
-        <v>2020</v>
-      </c>
-      <c r="J6" t="s">
+      <c r="M6" t="s">
         <v>72</v>
       </c>
-      <c r="K6" t="s">
+      <c r="N6" t="s">
         <v>73</v>
       </c>
-      <c r="L6" t="s">
-        <v>56</v>
-      </c>
-      <c r="M6" t="s">
-        <v>74</v>
-      </c>
-      <c r="N6" t="s">
-        <v>75</v>
-      </c>
-      <c r="O6" t="s">
-        <v>76</v>
-      </c>
     </row>
-    <row r="7" spans="1:20">
+    <row r="7" spans="1:19">
       <c r="A7">
         <v>5</v>
       </c>
       <c r="B7" t="s">
+        <v>74</v>
+      </c>
+      <c r="C7" t="s">
+        <v>34</v>
+      </c>
+      <c r="D7" t="s">
+        <v>75</v>
+      </c>
+      <c r="E7" t="s">
+        <v>48</v>
+      </c>
+      <c r="F7" t="s">
+        <v>76</v>
+      </c>
+      <c r="G7" t="s">
         <v>77</v>
       </c>
-      <c r="C7" t="s">
-        <v>36</v>
-      </c>
-      <c r="D7" t="s">
+      <c r="H7">
+        <v>2015</v>
+      </c>
+      <c r="I7" t="s">
         <v>78</v>
       </c>
-      <c r="E7" t="s">
-        <v>51</v>
-      </c>
-      <c r="G7" t="s">
+      <c r="J7" t="s">
+        <v>39</v>
+      </c>
+      <c r="K7" t="s">
+        <v>40</v>
+      </c>
+      <c r="L7" t="s">
         <v>79</v>
       </c>
-      <c r="H7" t="s">
+      <c r="M7" t="s">
+        <v>42</v>
+      </c>
+      <c r="N7" t="s">
         <v>80</v>
       </c>
-      <c r="I7">
-        <v>2015</v>
-      </c>
-      <c r="J7" t="s">
+      <c r="O7">
+        <v>120</v>
+      </c>
+      <c r="P7">
+        <v>19</v>
+      </c>
+      <c r="Q7">
+        <v>10</v>
+      </c>
+      <c r="R7" t="s">
+        <v>44</v>
+      </c>
+      <c r="S7" t="s">
         <v>81</v>
       </c>
-      <c r="K7" t="s">
-        <v>42</v>
-      </c>
-      <c r="L7" t="s">
-        <v>43</v>
-      </c>
-      <c r="M7" t="s">
-        <v>82</v>
-      </c>
-      <c r="N7" t="s">
-        <v>45</v>
-      </c>
-      <c r="O7" t="s">
-        <v>83</v>
-      </c>
-      <c r="P7">
-        <v>120</v>
-      </c>
-      <c r="Q7">
-        <v>19</v>
-      </c>
-      <c r="R7">
-        <v>10</v>
-      </c>
-      <c r="S7" t="s">
-        <v>47</v>
-      </c>
-      <c r="T7" t="s">
-        <v>84</v>
-      </c>
     </row>
-    <row r="8" spans="1:20">
+    <row r="8" spans="1:19">
       <c r="A8">
         <v>6</v>
       </c>
       <c r="B8" t="s">
+        <v>82</v>
+      </c>
+      <c r="C8" t="s">
+        <v>34</v>
+      </c>
+      <c r="D8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E8" t="s">
+        <v>48</v>
+      </c>
+      <c r="F8" t="s">
+        <v>84</v>
+      </c>
+      <c r="G8" t="s">
         <v>85</v>
       </c>
-      <c r="C8" t="s">
-        <v>36</v>
-      </c>
-      <c r="D8" t="s">
+      <c r="H8">
+        <v>2015</v>
+      </c>
+      <c r="I8" t="s">
         <v>86</v>
       </c>
-      <c r="E8" t="s">
-        <v>51</v>
-      </c>
-      <c r="G8" t="s">
+      <c r="J8" t="s">
+        <v>39</v>
+      </c>
+      <c r="K8" t="s">
+        <v>40</v>
+      </c>
+      <c r="L8" t="s">
         <v>87</v>
       </c>
-      <c r="H8" t="s">
+      <c r="M8" t="s">
+        <v>42</v>
+      </c>
+      <c r="N8" t="s">
         <v>88</v>
       </c>
-      <c r="I8">
-        <v>2015</v>
-      </c>
-      <c r="J8" t="s">
-        <v>89</v>
-      </c>
-      <c r="K8" t="s">
-        <v>42</v>
-      </c>
-      <c r="L8" t="s">
-        <v>43</v>
-      </c>
-      <c r="M8" t="s">
-        <v>90</v>
-      </c>
-      <c r="N8" t="s">
-        <v>45</v>
-      </c>
-      <c r="O8" t="s">
-        <v>91</v>
+      <c r="O8">
+        <v>154</v>
       </c>
       <c r="P8">
         <v>154</v>
       </c>
       <c r="Q8">
-        <v>154</v>
-      </c>
-      <c r="R8">
         <v>1</v>
       </c>
+      <c r="R8" t="s">
+        <v>44</v>
+      </c>
       <c r="S8" t="s">
-        <v>47</v>
-      </c>
-      <c r="T8" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
-    <row r="9" spans="1:20">
+    <row r="9" spans="1:19">
       <c r="A9">
         <v>7</v>
       </c>
       <c r="B9" t="s">
+        <v>90</v>
+      </c>
+      <c r="C9" t="s">
+        <v>34</v>
+      </c>
+      <c r="D9" t="s">
+        <v>91</v>
+      </c>
+      <c r="E9" t="s">
+        <v>48</v>
+      </c>
+      <c r="F9" t="s">
+        <v>92</v>
+      </c>
+      <c r="G9" t="s">
         <v>93</v>
       </c>
-      <c r="C9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D9" t="s">
+      <c r="H9">
+        <v>2024</v>
+      </c>
+      <c r="I9" t="s">
         <v>94</v>
       </c>
-      <c r="E9" t="s">
-        <v>51</v>
-      </c>
-      <c r="G9" t="s">
+      <c r="J9" t="s">
         <v>95</v>
       </c>
-      <c r="H9" t="s">
+      <c r="K9" t="s">
         <v>96</v>
       </c>
-      <c r="I9">
-        <v>2024</v>
-      </c>
-      <c r="J9" t="s">
+      <c r="L9" t="s">
         <v>97</v>
       </c>
-      <c r="K9" t="s">
+      <c r="M9" t="s">
         <v>98</v>
       </c>
-      <c r="L9" t="s">
+      <c r="N9" t="s">
         <v>99</v>
       </c>
-      <c r="M9" t="s">
-        <v>100</v>
-      </c>
-      <c r="N9" t="s">
-        <v>101</v>
-      </c>
-      <c r="O9" t="s">
-        <v>102</v>
-      </c>
     </row>
-    <row r="10" spans="1:20">
+    <row r="10" spans="1:19">
       <c r="A10">
         <v>8</v>
       </c>
       <c r="B10" t="s">
+        <v>100</v>
+      </c>
+      <c r="C10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" t="s">
+        <v>101</v>
+      </c>
+      <c r="E10" t="s">
+        <v>48</v>
+      </c>
+      <c r="F10" t="s">
+        <v>102</v>
+      </c>
+      <c r="G10" t="s">
         <v>103</v>
       </c>
-      <c r="C10" t="s">
-        <v>21</v>
-      </c>
-      <c r="D10" t="s">
+      <c r="H10">
+        <v>2019</v>
+      </c>
+      <c r="I10" t="s">
         <v>104</v>
       </c>
-      <c r="E10" t="s">
-        <v>51</v>
-      </c>
-      <c r="G10" t="s">
+      <c r="J10" t="s">
+        <v>52</v>
+      </c>
+      <c r="K10" t="s">
+        <v>53</v>
+      </c>
+      <c r="L10" t="s">
         <v>105</v>
       </c>
-      <c r="H10" t="s">
+      <c r="M10" t="s">
         <v>106</v>
       </c>
-      <c r="I10">
-        <v>2019</v>
-      </c>
-      <c r="J10" t="s">
+      <c r="N10" t="s">
         <v>107</v>
       </c>
-      <c r="K10" t="s">
-        <v>55</v>
-      </c>
-      <c r="L10" t="s">
-        <v>56</v>
-      </c>
-      <c r="M10" t="s">
-        <v>108</v>
-      </c>
-      <c r="N10" t="s">
-        <v>109</v>
-      </c>
-      <c r="O10" t="s">
-        <v>110</v>
-      </c>
     </row>
-    <row r="11" spans="1:20">
+    <row r="11" spans="1:19">
       <c r="A11">
         <v>9</v>
       </c>
       <c r="B11" t="s">
+        <v>108</v>
+      </c>
+      <c r="C11" t="s">
+        <v>20</v>
+      </c>
+      <c r="D11" t="s">
+        <v>109</v>
+      </c>
+      <c r="E11" t="s">
+        <v>48</v>
+      </c>
+      <c r="F11" t="s">
+        <v>110</v>
+      </c>
+      <c r="G11" t="s">
         <v>111</v>
       </c>
-      <c r="C11" t="s">
-        <v>21</v>
-      </c>
-      <c r="D11" t="s">
+      <c r="H11">
+        <v>2017</v>
+      </c>
+      <c r="I11" t="s">
         <v>112</v>
       </c>
-      <c r="E11" t="s">
-        <v>51</v>
-      </c>
-      <c r="G11" t="s">
+      <c r="J11" t="s">
         <v>113</v>
       </c>
-      <c r="H11" t="s">
+      <c r="K11" t="s">
         <v>114</v>
       </c>
-      <c r="I11">
-        <v>2017</v>
-      </c>
-      <c r="J11" t="s">
+      <c r="L11" t="s">
         <v>115</v>
       </c>
-      <c r="K11" t="s">
+      <c r="M11" t="s">
         <v>116</v>
       </c>
-      <c r="L11" t="s">
+      <c r="N11" t="s">
         <v>117</v>
-      </c>
-      <c r="M11" t="s">
-        <v>118</v>
-      </c>
-      <c r="N11" t="s">
-        <v>119</v>
-      </c>
-      <c r="O11" t="s">
-        <v>120</v>
       </c>
     </row>
   </sheetData>

</xml_diff>